<commit_message>
updated agenda - added GrowthHub session1
</commit_message>
<xml_diff>
--- a/unit-0/paneltalk-agenda/agenda.xlsx
+++ b/unit-0/paneltalk-agenda/agenda.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/git/Hdip2025/workshop-1-3/unit-0/paneltalk-agenda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222ABF27-1C60-1A4C-BE6A-153494C8EC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA2633E-C591-E147-9BC2-BEB91BCFD090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3440" yWindow="1060" windowWidth="31940" windowHeight="20420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2760" yWindow="500" windowWidth="33760" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1-1 - Workshop 1, 3 &amp; 5 -" sheetId="3" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Time</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Workshop Close_x000B_</t>
   </si>
   <si>
-    <t>GrowthHub</t>
-  </si>
-  <si>
     <t xml:space="preserve">Programming Lab - Siobhan, Mairead and Pete </t>
   </si>
   <si>
@@ -65,9 +62,6 @@
     <t xml:space="preserve"> Workshop 1, 3 &amp; 5 -January 10th 2025</t>
   </si>
   <si>
-    <t>More Information to follow</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Registration </t>
     </r>
@@ -105,31 +99,6 @@
         <family val="2"/>
       </rPr>
       <t>Laura (Auditorium)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color indexed="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Programme Overview - </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="14"/>
-        <color rgb="FFFEFEFE"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Eamonn and Frank (Auditorium)</t>
     </r>
     <r>
       <rPr>
@@ -343,6 +312,41 @@
  (F02)
 </t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Programme Overview - </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color rgb="FFFEFEFE"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Frank (Auditorium)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color indexed="12"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>The path to completion 
+GrowthHub</t>
+  </si>
+  <si>
+    <t>Dr Margaret Tynan</t>
+  </si>
+  <si>
+    <t>Registration (Auditorium)</t>
   </si>
 </sst>
 </file>
@@ -682,12 +686,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -697,15 +695,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -721,112 +710,127 @@
     <xf numFmtId="20" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2721,7 +2725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:F18"/>
+  <dimension ref="B1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
@@ -2729,214 +2733,223 @@
     <col min="3" max="3" width="11.33203125" style="1" customWidth="1"/>
     <col min="4" max="4" width="40.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="38.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="42.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="42.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" style="1" hidden="1" customWidth="1"/>
     <col min="8" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="2:7" ht="14" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C1" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="49"/>
+    </row>
+    <row r="2" spans="2:7" ht="43" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="2:6" ht="43" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="4" t="s">
+    <row r="3" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B3" s="5"/>
+      <c r="C3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B4" s="8"/>
+      <c r="C4" s="9">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>13</v>
       </c>
+      <c r="E4" s="47"/>
+      <c r="F4" s="10"/>
     </row>
-    <row r="3" spans="2:6" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B3" s="10"/>
-      <c r="C3" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>6</v>
-      </c>
+    <row r="5" spans="2:7" ht="46" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B5" s="11"/>
+      <c r="C5" s="9">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="47"/>
+      <c r="F5" s="12"/>
     </row>
-    <row r="4" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B4" s="13"/>
-      <c r="C4" s="14">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="D4" s="15" t="s">
+    <row r="6" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B6" s="11"/>
+      <c r="C6" s="9">
+        <v>0.4375</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="47"/>
+      <c r="F6" s="12"/>
+    </row>
+    <row r="7" spans="2:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B7" s="13"/>
+      <c r="C7" s="14">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="48"/>
+      <c r="F7" s="40" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="48"/>
+    </row>
+    <row r="8" spans="2:7" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B8" s="15"/>
+      <c r="C8" s="9">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="F8" s="44" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="5" spans="2:6" ht="46" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B5" s="18"/>
-      <c r="C5" s="14">
-        <v>0.42708333333333331</v>
-      </c>
-      <c r="D5" s="15" t="s">
+    <row r="9" spans="2:7" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B9" s="11"/>
+      <c r="C9" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="45"/>
+    </row>
+    <row r="10" spans="2:7" ht="50" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B10" s="11"/>
+      <c r="C10" s="9">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D10" s="27"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" ht="55" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B11" s="13"/>
+      <c r="C11" s="14">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D11" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+    </row>
+    <row r="12" spans="2:7" ht="41" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B12" s="11"/>
+      <c r="C12" s="9">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="34"/>
+      <c r="F12" s="37" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="38" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B13" s="11"/>
+      <c r="C13" s="9">
+        <v>44839.59375</v>
+      </c>
+      <c r="D13" s="35"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="38"/>
+    </row>
+    <row r="14" spans="2:7" ht="43" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B14" s="20"/>
+      <c r="C14" s="14">
+        <v>44839.614583333336</v>
+      </c>
+      <c r="D14" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="41"/>
+      <c r="F14" s="41"/>
+    </row>
+    <row r="15" spans="2:7" ht="89" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B15" s="11"/>
+      <c r="C15" s="9">
+        <v>44839.635416666664</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="42" t="s">
         <v>10</v>
-      </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="19"/>
-    </row>
-    <row r="6" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="18"/>
-      <c r="C6" s="14">
-        <v>0.4375</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="19"/>
-    </row>
-    <row r="7" spans="2:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B7" s="20"/>
-      <c r="C7" s="21">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" s="23"/>
-      <c r="F7" s="19"/>
-    </row>
-    <row r="8" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B8" s="24"/>
-      <c r="C8" s="14">
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B9" s="18"/>
-      <c r="C9" s="14">
-        <v>0.5</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="30"/>
-    </row>
-    <row r="10" spans="2:6" ht="50" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B10" s="18"/>
-      <c r="C10" s="14">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="D10" s="31"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="33" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" ht="55" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B11" s="20"/>
-      <c r="C11" s="21">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-    </row>
-    <row r="12" spans="2:6" ht="41" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B12" s="18"/>
-      <c r="C12" s="14">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="36"/>
-      <c r="F12" s="37" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" ht="38" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B13" s="18"/>
-      <c r="C13" s="14">
-        <v>44839.59375</v>
-      </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="40"/>
-    </row>
-    <row r="14" spans="2:6" ht="43" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B14" s="41"/>
-      <c r="C14" s="21">
-        <v>44839.614583333336</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-    </row>
-    <row r="15" spans="2:6" ht="89" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="18"/>
-      <c r="C15" s="14">
-        <v>44839.635416666664</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="42" t="s">
-        <v>11</v>
       </c>
       <c r="F15" s="43"/>
     </row>
-    <row r="16" spans="2:6" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="18"/>
-      <c r="C16" s="44">
+    <row r="16" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B16" s="11"/>
+      <c r="C16" s="21">
         <v>0.67708333333333337</v>
       </c>
-      <c r="D16" s="45"/>
-      <c r="E16" s="46" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="47"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="23"/>
     </row>
     <row r="17" spans="2:6" ht="55" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B17" s="18"/>
-      <c r="C17" s="44">
+      <c r="B17" s="11"/>
+      <c r="C17" s="21">
         <v>0.6875</v>
       </c>
-      <c r="D17" s="48" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="49"/>
-      <c r="F17" s="50"/>
+      <c r="D17" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="24"/>
+      <c r="F17" s="25"/>
     </row>
     <row r="18" spans="2:6" ht="38" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B18" s="6"/>
-      <c r="C18" s="5">
+      <c r="B18" s="4"/>
+      <c r="C18" s="3">
         <v>44839.708333333336</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="C1:D2"/>
     <mergeCell ref="E16:F17"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
@@ -2948,11 +2961,6 @@
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="F8:F9"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="C1:D2"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup scale="70" orientation="portrait"/>

</xml_diff>